<commit_message>
pkg data download working now
</commit_message>
<xml_diff>
--- a/data/raw/raw-sunburst-fig-data-from-jon-new.xlsx
+++ b/data/raw/raw-sunburst-fig-data-from-jon-new.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\au757887\PC_documents\_git-it\pietool\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05532978-30B4-4CB7-B572-A06E174326FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F75B95E-FCF9-4F72-A98F-B90B6856B56B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6E41958F-17C1-4081-8916-3DF7BBE757A7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{78D5E249-EDAF-420B-97EF-4D4101A6EF6C}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
+    <sheet name="pesticide_load_table_2026-07-25" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t>Substance</t>
   </si>
@@ -28,7 +28,7 @@
     <t>Substance_ToxIndex</t>
   </si>
   <si>
-    <t>Substance_SocietalCostIndex</t>
+    <t>Substance_CostIndex</t>
   </si>
   <si>
     <t>ecotoxicity_aquatic_load</t>
@@ -43,6 +43,18 @@
     <t>human_health_load</t>
   </si>
   <si>
+    <t>ecotoxicity_aquatic_cost</t>
+  </si>
+  <si>
+    <t>ecotoxicity_terrestrial_cost</t>
+  </si>
+  <si>
+    <t>environmental_fate_cost</t>
+  </si>
+  <si>
+    <t>human_health_cost</t>
+  </si>
+  <si>
     <t>QuantAppl_kgperarea</t>
   </si>
   <si>
@@ -58,6 +70,18 @@
     <t>HumHea_Load</t>
   </si>
   <si>
+    <t>EcoAqu_Cost</t>
+  </si>
+  <si>
+    <t>EcoTerr_Cost</t>
+  </si>
+  <si>
+    <t>EnvPers_Cost</t>
+  </si>
+  <si>
+    <t>HumHea_Cost</t>
+  </si>
+  <si>
     <t>Total_Load</t>
   </si>
   <si>
@@ -74,15 +98,66 @@
   </si>
   <si>
     <t>MCPA</t>
+  </si>
+  <si>
+    <t>1,914</t>
+  </si>
+  <si>
+    <t>19,333</t>
+  </si>
+  <si>
+    <t>1,306</t>
+  </si>
+  <si>
+    <t>2,558</t>
+  </si>
+  <si>
+    <t>2,461</t>
+  </si>
+  <si>
+    <t>1,806</t>
+  </si>
+  <si>
+    <t>20,218</t>
+  </si>
+  <si>
+    <t>2,093</t>
+  </si>
+  <si>
+    <t>6,739</t>
+  </si>
+  <si>
+    <t>10,629</t>
+  </si>
+  <si>
+    <t>12,542</t>
+  </si>
+  <si>
+    <t>2,499</t>
+  </si>
+  <si>
+    <t>1,913</t>
+  </si>
+  <si>
+    <t>2,667</t>
+  </si>
+  <si>
+    <t>1,279</t>
+  </si>
+  <si>
+    <t>1,131</t>
+  </si>
+  <si>
+    <t>5,117</t>
+  </si>
+  <si>
+    <t>4,922</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.000"/>
-  </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -562,7 +637,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -937,11 +1012,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B102C799-78D7-4593-B6E7-9E352EA8D196}">
-  <dimension ref="A1:N5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D618E7C9-6E99-491B-9D09-5D217C44F706}">
+  <dimension ref="A1:V5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -984,10 +1059,34 @@
       <c r="N1" t="s">
         <v>13</v>
       </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B2" s="1">
         <v>0.377</v>
@@ -1008,30 +1107,54 @@
         <v>0.23499999999999999</v>
       </c>
       <c r="H2" s="1">
+        <v>0.156</v>
+      </c>
+      <c r="I2" s="1">
+        <v>0.69799999999999995</v>
+      </c>
+      <c r="J2" s="1">
+        <v>3.71</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L2" s="1">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="M2" s="1">
         <v>0.69399999999999995</v>
       </c>
-      <c r="J2" s="1">
+      <c r="N2" s="1">
         <v>0.85699999999999998</v>
       </c>
-      <c r="K2" s="1">
-        <v>1.9139999999999999</v>
-      </c>
-      <c r="L2" s="1">
+      <c r="O2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="P2" s="1">
         <v>0.70399999999999996</v>
       </c>
-      <c r="M2" s="1">
-        <v>1.131</v>
-      </c>
-      <c r="N2" s="1">
-        <v>19.332999999999998</v>
+      <c r="Q2" s="1">
+        <v>0.46700000000000003</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="S2" s="1">
+        <v>11.13</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B3" s="1">
         <v>0.38400000000000001</v>
@@ -1052,30 +1175,54 @@
         <v>0.37</v>
       </c>
       <c r="H3" s="1">
+        <v>0.26700000000000002</v>
+      </c>
+      <c r="I3" s="1">
+        <v>0.748</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="L3" s="1">
         <v>2E-3</v>
-      </c>
-      <c r="I3" s="1">
-        <v>1E-3</v>
-      </c>
-      <c r="J3" s="1">
-        <v>1E-3</v>
-      </c>
-      <c r="K3" s="1">
-        <v>1E-3</v>
-      </c>
-      <c r="L3" s="1">
-        <v>1E-3</v>
       </c>
       <c r="M3" s="1">
         <v>1E-3</v>
       </c>
       <c r="N3" s="1">
+        <v>1E-3</v>
+      </c>
+      <c r="O3" s="1">
+        <v>1E-3</v>
+      </c>
+      <c r="P3" s="1">
+        <v>1E-3</v>
+      </c>
+      <c r="Q3" s="1">
+        <v>1E-3</v>
+      </c>
+      <c r="R3" s="1">
+        <v>1E-3</v>
+      </c>
+      <c r="S3" s="1">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="T3" s="1">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="U3" s="1">
+        <v>1E-3</v>
+      </c>
+      <c r="V3" s="1">
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B4" s="1">
         <v>0.47299999999999998</v>
@@ -1096,36 +1243,60 @@
         <v>0.437</v>
       </c>
       <c r="H4" s="1">
+        <v>0.66300000000000003</v>
+      </c>
+      <c r="I4" s="1">
+        <v>0.78900000000000003</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="L4" s="1">
         <v>0.14399999999999999</v>
       </c>
-      <c r="I4" s="1">
+      <c r="M4" s="1">
         <v>0.14199999999999999</v>
       </c>
-      <c r="J4" s="1">
+      <c r="N4" s="1">
         <v>4.7E-2</v>
       </c>
-      <c r="K4" s="1">
+      <c r="O4" s="1">
         <v>4.7E-2</v>
       </c>
-      <c r="L4" s="1">
+      <c r="P4" s="1">
         <v>6.3E-2</v>
       </c>
-      <c r="M4" s="1">
+      <c r="Q4" s="1">
+        <v>9.5000000000000001E-2</v>
+      </c>
+      <c r="R4" s="1">
+        <v>0.114</v>
+      </c>
+      <c r="S4" s="1">
+        <v>0.27600000000000002</v>
+      </c>
+      <c r="T4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U4" s="1">
         <v>6.8000000000000005E-2</v>
       </c>
-      <c r="N4" s="1">
-        <v>1.306</v>
+      <c r="V4" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="B5" s="1">
         <v>0.32400000000000001</v>
       </c>
-      <c r="C5" s="1">
-        <v>5.117</v>
+      <c r="C5" s="1" t="s">
+        <v>42</v>
       </c>
       <c r="D5" s="1">
         <v>0.159</v>
@@ -1140,25 +1311,49 @@
         <v>0.17100000000000001</v>
       </c>
       <c r="H5" s="1">
+        <v>0.107</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L5" s="1">
         <v>0.5</v>
       </c>
-      <c r="I5" s="1">
+      <c r="M5" s="1">
         <v>7.9000000000000001E-2</v>
       </c>
-      <c r="J5" s="1">
+      <c r="N5" s="1">
         <v>0.26200000000000001</v>
       </c>
-      <c r="K5" s="1">
+      <c r="O5" s="1">
         <v>0.22900000000000001</v>
       </c>
-      <c r="L5" s="1">
+      <c r="P5" s="1">
         <v>8.5999999999999993E-2</v>
       </c>
-      <c r="M5" s="1">
+      <c r="Q5" s="1">
+        <v>5.2999999999999999E-2</v>
+      </c>
+      <c r="R5" s="1">
+        <v>0.63900000000000001</v>
+      </c>
+      <c r="S5" s="1">
+        <v>1334</v>
+      </c>
+      <c r="T5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="U5" s="1">
         <v>0.16200000000000001</v>
       </c>
-      <c r="N5" s="1">
-        <v>2.5579999999999998</v>
+      <c r="V5" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sub clrs same order
</commit_message>
<xml_diff>
--- a/data/raw/raw-sunburst-fig-data-from-jon-new.xlsx
+++ b/data/raw/raw-sunburst-fig-data-from-jon-new.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\au757887\PC_documents\_git-it\pietool\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F75B95E-FCF9-4F72-A98F-B90B6856B56B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DF4379F-8F62-43D4-8453-B5B18A2EF773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{78D5E249-EDAF-420B-97EF-4D4101A6EF6C}"/>
   </bookViews>
@@ -1017,75 +1017,75 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B2" s="1">
@@ -1153,7 +1153,7 @@
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B3" s="1">
@@ -1221,7 +1221,7 @@
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B4" s="1">
@@ -1289,7 +1289,7 @@
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B5" s="1">

</xml_diff>